<commit_message>
Fix: Excel sync now supports adding single users without affecting others (Upsert logic)
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Linoy\Desktop\עזרה ורפואה\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{7EBD4EB0-F4BC-4995-AF50-B0522EC7D1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B8A20CB2-485D-4D58-852C-B3AA0404D611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0774DACE-2576-4EE6-9185-46D6F144DF80}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="8964" windowHeight="8880" xr2:uid="{0774DACE-2576-4EE6-9185-46D6F144DF80}"/>
   </bookViews>
   <sheets>
     <sheet name="users-template" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="8" uniqueCount="8">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="4" uniqueCount="4">
   <si>
     <t>username</t>
   </si>
@@ -33,22 +33,10 @@
     <t>password</t>
   </si>
   <si>
-    <t>admin</t>
+    <t>oron</t>
   </si>
   <si>
-    <t>admin123</t>
-  </si>
-  <si>
-    <t>student1</t>
-  </si>
-  <si>
-    <t>student123</t>
-  </si>
-  <si>
-    <t>linoyezra</t>
-  </si>
-  <si>
-    <t>yizhak</t>
+    <t>oron123</t>
   </si>
 </sst>
 </file>
@@ -927,7 +915,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FFBAB83-69E1-4352-922B-0ECE6F044901}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -946,30 +934,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4">
-        <v>214215444</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5">
-        <v>207067091</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: ensure webhook API endpoints are correctly mounted and exposed
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Linoy\Desktop\עזרה ורפואה\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B8A20CB2-485D-4D58-852C-B3AA0404D611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B6F6D29D-0FED-4E80-85A8-4ED10BE509EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2688" yWindow="2688" windowWidth="8964" windowHeight="8880" xr2:uid="{0774DACE-2576-4EE6-9185-46D6F144DF80}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="4" uniqueCount="4">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5" uniqueCount="5">
   <si>
     <t>username</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t>oron123</t>
+  </si>
+  <si>
+    <t>course_group_id</t>
   </si>
 </sst>
 </file>
@@ -915,18 +918,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FFBAB83-69E1-4352-922B-0ECE6F044901}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -936,5 +942,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="257" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>